<commit_message>
Descuento por producto: columna en la planilla, precios y mensajes
- Excel: columna `descuento` (% entero, 0-90) entre cantidades y activo,
  con validación e instrucciones en la hoja leeme.
- index.html: lee `descuento` por nombre, calcula el precio rebajado
  (redondeo a $10) y lo muestra en su misma caja: lista tachada + burbuja
  -N% sobre el precio nuevo, en tarjetas, ficha y carrito. La fila sigue
  en 42px. WhatsApp/Instagram llevan precio nuevo y anterior; el carrito
  suma el ahorro.
- LEEME: nota sobre fotos en Cloudinary.
- mockups: propuestas de diseño del descuento.
- .gitignore: _to_delete/

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y8G65uwrp8bGAftV2ZQfcf
</commit_message>
<xml_diff>
--- a/catalogo_heart_graphic.xlsx
+++ b/catalogo_heart_graphic.xlsx
@@ -127,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -181,6 +181,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -256,6 +265,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Heart Graphic</author>
+  </authors>
+  <commentList>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>% de descuento por defecto del producto (0–90). 0 o vacío = sin descuento. Se aplica a todos los tramos de 'cantidades' y en la web se ve el precio viejo tachado y el nuevo.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -547,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -561,6 +585,8 @@
     <col width="56" customWidth="1" min="9" max="9"/>
     <col width="64" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -619,7 +645,12 @@
           <t>cantidades</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="20" t="inlineStr">
+        <is>
+          <t>descuento</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>activo</t>
         </is>
@@ -676,7 +707,10 @@
 }</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -729,7 +763,10 @@
 }</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr">
+      <c r="L3" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -781,7 +818,10 @@
 }</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -832,7 +872,10 @@
 }</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr">
+      <c r="L5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -883,7 +926,10 @@
 }</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -934,7 +980,10 @@
 }</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr">
+      <c r="L7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -985,7 +1034,10 @@
 }</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1038,7 +1090,10 @@
 }</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr">
+      <c r="L9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1089,7 +1144,10 @@
 }</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1135,7 +1193,10 @@
 }</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr">
+      <c r="L11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1185,7 +1246,10 @@
 }</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1233,7 +1297,10 @@
           <t>[{"unidades":10, "precio":5000}, {"unidades":20, "precio":8600}, {"unidades":30, "precio":11100}, {"unidades":50, "precio":15000}, {"unidades":100, "precio":26000}]</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr">
+      <c r="L13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1281,7 +1348,10 @@
           <t>[{"unidades":1, "precio":3000}, {"unidades":10, "precio":25000}, {"unidades":20, "precio":40000}, {"unidades":30, "precio":53000}]</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1329,7 +1399,10 @@
           <t>[{"unidades":1, "precio":3000}, {"unidades":2, "precio":5000}]</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr">
+      <c r="L15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1377,7 +1450,10 @@
           <t>[{"unidades":1, "precio":3000}, {"unidades":2, "precio":5000}]</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1429,7 +1505,10 @@
 }</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr">
+      <c r="L17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1479,7 +1558,10 @@
 }</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1529,7 +1611,10 @@
 }</t>
         </is>
       </c>
-      <c r="L19" s="7" t="inlineStr">
+      <c r="L19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1575,7 +1660,10 @@
 }</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1619,7 +1707,10 @@
           <t>[{"unidades":1, "precio":3000}, {"unidades":2, "precio":5000}, {"unidades":3, "precio":6000}]</t>
         </is>
       </c>
-      <c r="L21" s="7" t="inlineStr">
+      <c r="L21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1669,7 +1760,10 @@
 }</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="L22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1720,14 +1814,24 @@
 }</t>
         </is>
       </c>
-      <c r="L23" s="7" t="inlineStr">
+      <c r="L23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="L2:L200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Descuento" error="Escribe un número entero entre 0 y 90 (es un porcentaje)." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>90</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1737,7 +1841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A64"/>
+  <dimension ref="A1:A70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -2116,36 +2220,71 @@
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t>Los precios salen SOLO de la columna 'cantidades'. No hay hoja de respaldo.</t>
+          <t>• descuento: porcentaje de descuento POR DEFECTO del producto (número entero, sin el signo %). Ej: 15</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Si una celda 'cantidades' queda mal escrita, ese producto NO aparece en la web y el aviso sale en la consola del navegador (F12).</t>
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Se aplica a TODOS los tramos de 'cantidades' del producto. En la web se ve el precio viejo tachado,</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="14" t="inlineStr"/>
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  el precio nuevo y la etiqueta -15%. El precio nuevo se redondea a los $10 más cercanos.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="15" t="inlineStr">
-        <is>
-          <t>IMPORTANTE: no cambiar los nombres de las hojas ni de las columnas (la primera fila).</t>
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  El mensaje de WhatsApp/Instagram también lleva el precio con descuento (y el precio anterior).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">
         <is>
+          <t xml:space="preserve">  0 o vacío = sin descuento (se muestra el precio normal, sin tachar nada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="inlineStr">
+        <is>
+          <t>Los precios salen SOLO de la columna 'cantidades'. No hay hoja de respaldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Si una celda 'cantidades' queda mal escrita, ese producto NO aparece en la web y el aviso sale en la consola del navegador (F12).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>IMPORTANTE: no cambiar los nombres de las hojas ni de las columnas (la primera fila).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
           <t>El orden de las columnas sí puede cambiar: la web las busca por su nombre.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="14" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
         <is>
           <t>Todas las fotos van por URL completa (https://...). No se usan archivos locales.</t>
         </is>

</xml_diff>

<commit_message>
Plantilla del catalogo: columna tarjeta_inicio
Columna nueva en la hoja productos (lista si/no) y su explicacion en leeme:
marca que productos rotan en la tarjeta de la entrada salud.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalogo_heart_graphic.xlsx
+++ b/catalogo_heart_graphic.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -587,6 +587,7 @@
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -653,6 +654,11 @@
       <c r="M1" s="1" t="inlineStr">
         <is>
           <t>activo</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>tarjeta_inicio</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1830,10 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="N2:N200" type="list" allowBlank="1" showErrorMessage="1" errorTitle="tarjeta_inicio" error="Escribe si o no.">
+      <formula1>"si,no"</formula1>
+    </dataValidation>
     <dataValidation sqref="L2:L200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Descuento" error="Escribe un número entero entre 0 y 90 (es un porcentaje)." type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>90</formula2>
@@ -1841,7 +1850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A70"/>
+  <dimension ref="A1:A74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -2290,6 +2299,30 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• tarjeta_inicio: 'si' = el producto rota en la tarjeta grande de la ENTRADA SALUD (inicio de la página).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Solo afecta esa tarjeta: no cambia el carrusel ni los demás destacados. Vacío o 'no' = no aparece en ella.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Si ningún producto tiene 'si', la tarjeta rota por todo el catálogo. Los planners no entran (tienen su propia planilla).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>